<commit_message>
Updated for test 6 SE
</commit_message>
<xml_diff>
--- a/latest/Spike-SysML Summary.xlsx
+++ b/latest/Spike-SysML Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jarret\Documents\GitHub\Spike-SysML\development\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A8F30E5-4920-4703-9A41-6193FDC5E970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDF0408-A518-447B-82E3-B77BDFA882C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
+    <workbookView xWindow="34452" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Cal Runs</t>
   </si>
@@ -83,21 +83,6 @@
     <t>5 Freestyle</t>
   </si>
   <si>
-    <t>Op Run 2</t>
-  </si>
-  <si>
-    <t>Op Run 1</t>
-  </si>
-  <si>
-    <t>Op Run 3</t>
-  </si>
-  <si>
-    <t>Op Run 4</t>
-  </si>
-  <si>
-    <t>Op Run 5</t>
-  </si>
-  <si>
     <t>Words</t>
   </si>
   <si>
@@ -117,6 +102,9 @@
   </si>
   <si>
     <t>Error</t>
+  </si>
+  <si>
+    <t>6 SE</t>
   </si>
 </sst>
 </file>
@@ -175,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -195,12 +183,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -237,652 +228,6 @@
     <c:autoTitleDeleted val="1"/>
     <c:plotArea>
       <c:layout/>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$D$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>4 Freestyle</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent2"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$16:$B$27</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="7">
-                  <c:v>Op Run 1</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Op Run 2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Op Run 3</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Op Run 4</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Op Run 5</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$D$16:$D$27</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="4" formatCode="General">
-                  <c:v>395</c:v>
-                </c:pt>
-                <c:pt idx="5" formatCode="General">
-                  <c:v>33</c:v>
-                </c:pt>
-                <c:pt idx="6" formatCode="General">
-                  <c:v>38</c:v>
-                </c:pt>
-                <c:pt idx="7" formatCode="General">
-                  <c:v>99</c:v>
-                </c:pt>
-                <c:pt idx="8" formatCode="General">
-                  <c:v>87</c:v>
-                </c:pt>
-                <c:pt idx="9" formatCode="General">
-                  <c:v>95</c:v>
-                </c:pt>
-                <c:pt idx="10" formatCode="General">
-                  <c:v>81</c:v>
-                </c:pt>
-                <c:pt idx="11" formatCode="General">
-                  <c:v>97</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-7A11-48B6-B1E1-5B8446750985}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$F$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>5 Freestyle</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent4"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$F$16:$F$27</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="2">
-                  <c:v>228</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>78</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>191</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>178</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>201</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>193</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>257</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>183</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>256</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>180</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-7A11-48B6-B1E1-5B8446750985}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>4 SE</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$16:$B$27</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="7">
-                  <c:v>Op Run 1</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Op Run 2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Op Run 3</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Op Run 4</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Op Run 5</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$C$16:$C$27</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
-                  <c:v>314</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>359</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>641</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>409</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>366</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>469</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>173</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>197</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>171</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>198</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>196</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>200</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-7A11-48B6-B1E1-5B8446750985}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$E$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>5 SE</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent3"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$16:$B$27</c:f>
-              <c:strCache>
-                <c:ptCount val="12"/>
-                <c:pt idx="7">
-                  <c:v>Op Run 1</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>Op Run 2</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>Op Run 3</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>Op Run 4</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>Op Run 5</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$E$16:$E$27</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="2" formatCode="General">
-                  <c:v>442</c:v>
-                </c:pt>
-                <c:pt idx="3" formatCode="General">
-                  <c:v>689</c:v>
-                </c:pt>
-                <c:pt idx="4" formatCode="General">
-                  <c:v>479</c:v>
-                </c:pt>
-                <c:pt idx="5" formatCode="General">
-                  <c:v>264</c:v>
-                </c:pt>
-                <c:pt idx="6" formatCode="General">
-                  <c:v>74</c:v>
-                </c:pt>
-                <c:pt idx="7" formatCode="General">
-                  <c:v>72</c:v>
-                </c:pt>
-                <c:pt idx="8" formatCode="General">
-                  <c:v>71</c:v>
-                </c:pt>
-                <c:pt idx="9" formatCode="General">
-                  <c:v>62</c:v>
-                </c:pt>
-                <c:pt idx="10" formatCode="General">
-                  <c:v>72</c:v>
-                </c:pt>
-                <c:pt idx="11" formatCode="General">
-                  <c:v>77</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-7A11-48B6-B1E1-5B8446750985}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:smooth val="0"/>
-        <c:axId val="1430609439"/>
-        <c:axId val="1430609919"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="1430609439"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="low"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1430609919"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:tickMarkSkip val="1"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="1430609919"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="65000"/>
-                        <a:lumOff val="35000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>Distance</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" baseline="0"/>
-                  <a:t> to wall (mm)</a:t>
-                </a:r>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1430609439"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:autoTitleDeleted val="1"/>
-    <c:plotArea>
-      <c:layout/>
       <c:barChart>
         <c:barDir val="col"/>
         <c:grouping val="clustered"/>
@@ -974,7 +319,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent4"/>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1045,7 +392,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent6"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1116,7 +463,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent3"/>
+              <a:srgbClr val="00B0F0"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1168,6 +515,59 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-B31A-4E47-A125-2957C3653DEA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$G$5:$G$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1C6B-4A7D-8E9A-CBC3F1217CFE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1374,7 +774,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1496,7 +896,9 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent4"/>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1581,7 +983,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent6"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1666,7 +1068,7 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent3"/>
+              <a:srgbClr val="00B0F0"/>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1732,6 +1134,88 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000002-3983-4C49-A73A-06B1D29DCB9D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="4"/>
+              <c:pt idx="0">
+                <c:v>Op Avg Dist</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Max-Min</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Sdev</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Error</c:v>
+              </c:pt>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:autoCat val="1"/>
+                </c:ext>
+              </c:extLst>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet1!$G$9:$G$15</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Sheet1!$G$11:$G$13,Sheet1!$G$15)</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.0498447189992426</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>104</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-D6E6-4A6C-8AC9-E6D23C79F65F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1938,6 +1422,635 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>4 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$B$16:$B$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$16:$C$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>314</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>359</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>641</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>409</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>366</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>469</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>173</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>197</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>171</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>196</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-8D7E-4F84-BBD3-152429E7606B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$E$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$B$16:$B$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$E$16:$E$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>442</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>689</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>479</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>264</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>62</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>77</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000A-8D7E-4F84-BBD3-152429E7606B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$G$16:$G$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>533</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>498</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>530</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>138</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>148</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>157</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>147</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>156</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000B-8D7E-4F84-BBD3-152429E7606B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>4 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$B$16:$B$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$D$16:$D$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>395</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>97</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000006-8D7E-4F84-BBD3-152429E7606B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$F$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$F$16:$F$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>228</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>191</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>178</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>201</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>193</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>257</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>183</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>180</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-8D7E-4F84-BBD3-152429E7606B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1430609439"/>
+        <c:axId val="1430609919"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1430609439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1430609919"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:tickMarkSkip val="1"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1430609919"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Distance</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> to wall (mm)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1430609439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2018,48 +2131,8 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -2086,8 +2159,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2188,7 +2261,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="19050" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -2220,10 +2293,10 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -2263,23 +2336,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
         </a:schemeClr>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
             <a:lumMod val="65000"/>
             <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -2384,8 +2456,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -2517,20 +2589,19 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="lt1"/>
       </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -2544,17 +2615,6 @@
         <a:lumOff val="35000"/>
       </a:schemeClr>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -3077,530 +3137,27 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>486276</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>75635</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>123206</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>166234</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>53788</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>134470</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="4" name="Chart 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D8F885CD-BFFF-F0D2-E3D5-13DB673A434E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{616FD840-7DC9-A323-C601-D3C1664B55FD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3620,27 +3177,29 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>311687</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>54909</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>366428</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>16753</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>55694</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>134471</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
+        <xdr:cNvPr id="5" name="Chart 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{616FD840-7DC9-A323-C601-D3C1664B55FD}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F4C806B-8AF9-498A-9CF9-59D8E5CB173A}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="0"/>
@@ -3656,23 +3215,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>253361</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>145786</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>305245</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>101916</xdr:rowOff>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>516703</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 4">
+        <xdr:cNvPr id="6" name="Chart 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F4C806B-8AF9-498A-9CF9-59D8E5CB173A}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C6906456-FC7D-4DBE-A0A2-536E88359AED}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4012,7 +3571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22FC483D-A2EB-4AB5-93A8-361DFBAB7337}">
-  <dimension ref="B2:F30"/>
+  <dimension ref="B2:H30"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.3984375" customWidth="1"/>
@@ -4021,43 +3580,53 @@
     <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" customWidth="1"/>
+    <col min="8" max="8" width="2.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="2.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="G2" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="7">
+        <v>16</v>
+      </c>
+      <c r="C3" s="11">
         <v>46199</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="11">
         <v>46200</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="11">
         <v>46201</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="11">
         <v>46202</v>
       </c>
+      <c r="G3" s="11">
+        <v>46203</v>
+      </c>
+      <c r="H3" s="10"/>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -4073,8 +3642,12 @@
       <c r="F4" s="3">
         <v>6</v>
       </c>
+      <c r="G4" s="3">
+        <v>3</v>
+      </c>
+      <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
@@ -4090,8 +3663,12 @@
       <c r="F5" s="3">
         <v>0</v>
       </c>
+      <c r="G5" s="3">
+        <v>3</v>
+      </c>
+      <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
@@ -4107,8 +3684,12 @@
       <c r="F6" s="3">
         <v>0</v>
       </c>
+      <c r="G6" s="3">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3"/>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
@@ -4124,29 +3705,38 @@
       <c r="F7" s="3">
         <v>0</v>
       </c>
+      <c r="G7" s="3">
+        <v>2</v>
+      </c>
+      <c r="H7" s="3"/>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="8">
+        <v>17</v>
+      </c>
+      <c r="C8" s="7">
         <f>C7+C4</f>
         <v>9</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="7">
         <f>D7+D4</f>
         <v>8</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="7">
         <f>E7+E4</f>
         <v>6</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="7">
         <f>F7+F4</f>
         <v>6</v>
       </c>
+      <c r="G8" s="7">
+        <f>G7+G4</f>
+        <v>5</v>
+      </c>
+      <c r="H8" s="3"/>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
@@ -4162,8 +3752,12 @@
       <c r="F9" s="4">
         <v>180</v>
       </c>
+      <c r="G9" s="4">
+        <v>135</v>
+      </c>
+      <c r="H9" s="4"/>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
@@ -4179,8 +3773,12 @@
       <c r="F10" s="4">
         <v>257</v>
       </c>
+      <c r="G10" s="4">
+        <v>157</v>
+      </c>
+      <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
@@ -4196,8 +3794,12 @@
       <c r="F11" s="4">
         <v>213.8</v>
       </c>
+      <c r="G11" s="4">
+        <v>148</v>
+      </c>
+      <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B12" s="1" t="s">
         <v>7</v>
       </c>
@@ -4213,27 +3815,35 @@
       <c r="F12" s="5">
         <v>77</v>
       </c>
+      <c r="G12" s="5">
+        <v>22</v>
+      </c>
+      <c r="H12" s="5"/>
     </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="9">
         <v>10.781465577554844</v>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="9">
         <v>6.7646138101151054</v>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="9">
         <v>4.8744230427815767</v>
       </c>
-      <c r="F13" s="10">
+      <c r="F13" s="9">
         <v>35.130613430454076</v>
       </c>
+      <c r="G13" s="9">
+        <v>8.0498447189992426</v>
+      </c>
+      <c r="H13" s="5"/>
     </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B14" s="1" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C14" s="5">
         <v>189</v>
@@ -4247,204 +3857,239 @@
       <c r="F14" s="5">
         <v>55</v>
       </c>
+      <c r="G14" s="5">
+        <v>44</v>
+      </c>
+      <c r="H14" s="5"/>
     </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="10">
+        <v>20</v>
+      </c>
+      <c r="C15" s="9">
         <f>C11-C14</f>
         <v>3.4000000000000057</v>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="9">
         <f>D11-D14</f>
         <v>26.399999999999991</v>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="9">
         <f>E11-E14</f>
         <v>-7.2000000000000028</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="9">
         <f>F11-F14</f>
         <v>158.80000000000001</v>
       </c>
+      <c r="G15" s="9">
+        <f>G11-G14</f>
+        <v>104</v>
+      </c>
+      <c r="H15" s="5"/>
     </row>
-    <row r="16" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B16" s="1"/>
       <c r="C16" s="2">
         <v>314</v>
       </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="2"/>
+      <c r="D16" s="2">
+        <v>395</v>
+      </c>
+      <c r="E16" s="2">
+        <v>442</v>
+      </c>
+      <c r="F16" s="2">
+        <v>228</v>
+      </c>
+      <c r="G16" s="3">
+        <v>533</v>
+      </c>
+      <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B17" s="1"/>
       <c r="C17" s="2">
         <v>359</v>
       </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="2"/>
+      <c r="D17" s="2">
+        <v>33</v>
+      </c>
+      <c r="E17" s="2">
+        <v>689</v>
+      </c>
+      <c r="F17" s="2">
+        <v>78</v>
+      </c>
+      <c r="G17" s="3">
+        <v>498</v>
+      </c>
+      <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B18" s="1"/>
       <c r="C18" s="2">
         <v>641</v>
       </c>
+      <c r="D18" s="2">
+        <v>38</v>
+      </c>
       <c r="E18" s="2">
-        <v>442</v>
+        <v>479</v>
       </c>
       <c r="F18" s="2">
-        <v>228</v>
-      </c>
+        <v>191</v>
+      </c>
+      <c r="G18" s="3">
+        <v>530</v>
+      </c>
+      <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B19" s="1"/>
       <c r="C19" s="2">
         <v>409</v>
       </c>
-      <c r="D19" s="2"/>
+      <c r="D19" s="2">
+        <v>99</v>
+      </c>
       <c r="E19" s="2">
-        <v>689</v>
+        <v>264</v>
       </c>
       <c r="F19" s="2">
-        <v>78</v>
-      </c>
+        <v>178</v>
+      </c>
+      <c r="G19" s="3">
+        <v>138</v>
+      </c>
+      <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B20" s="1"/>
       <c r="C20" s="2">
         <v>366</v>
       </c>
       <c r="D20" s="2">
-        <v>395</v>
+        <v>87</v>
       </c>
       <c r="E20" s="2">
-        <v>479</v>
+        <v>74</v>
       </c>
       <c r="F20" s="2">
-        <v>191</v>
+        <v>201</v>
+      </c>
+      <c r="G20" s="3">
+        <v>148</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B21" s="1"/>
       <c r="C21" s="2">
         <v>469</v>
       </c>
       <c r="D21" s="2">
-        <v>33</v>
+        <v>95</v>
       </c>
       <c r="E21" s="2">
-        <v>264</v>
+        <v>72</v>
       </c>
       <c r="F21" s="2">
-        <v>178</v>
+        <v>193</v>
+      </c>
+      <c r="G21" s="3">
+        <v>157</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B22" s="1"/>
       <c r="C22" s="2">
         <v>173</v>
       </c>
       <c r="D22" s="2">
-        <v>38</v>
+        <v>81</v>
       </c>
       <c r="E22" s="2">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F22" s="2">
-        <v>201</v>
+        <v>257</v>
+      </c>
+      <c r="G22" s="3">
+        <v>135</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B23" s="1" t="s">
-        <v>15</v>
-      </c>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B23" s="1"/>
       <c r="C23" s="2">
         <v>197</v>
       </c>
       <c r="D23" s="2">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E23" s="2">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F23" s="2">
-        <v>193</v>
-      </c>
+        <v>183</v>
+      </c>
+      <c r="G23" s="3">
+        <v>145</v>
+      </c>
+      <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B24" s="1" t="s">
-        <v>14</v>
-      </c>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B24" s="1"/>
       <c r="C24" s="2">
         <v>171</v>
       </c>
-      <c r="D24" s="2">
-        <v>87</v>
-      </c>
       <c r="E24" s="2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F24" s="2">
-        <v>257</v>
-      </c>
+        <v>256</v>
+      </c>
+      <c r="G24" s="3">
+        <v>147</v>
+      </c>
+      <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B25" s="1" t="s">
-        <v>16</v>
-      </c>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B25" s="1"/>
       <c r="C25" s="2">
         <v>198</v>
       </c>
-      <c r="D25" s="2">
-        <v>95</v>
-      </c>
       <c r="E25" s="2">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="F25" s="2">
-        <v>183</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="G25" s="3">
+        <v>156</v>
+      </c>
+      <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B26" s="1" t="s">
-        <v>17</v>
-      </c>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B26" s="1"/>
       <c r="C26" s="2">
         <v>196</v>
       </c>
-      <c r="D26" s="2">
-        <v>81</v>
-      </c>
-      <c r="E26" s="2">
-        <v>72</v>
-      </c>
-      <c r="F26" s="2">
-        <v>256</v>
-      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B27" s="1" t="s">
-        <v>18</v>
-      </c>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B27" s="1"/>
       <c r="C27" s="6">
         <v>200</v>
       </c>
-      <c r="D27" s="6">
-        <v>97</v>
-      </c>
-      <c r="E27" s="6">
-        <v>77</v>
-      </c>
-      <c r="F27" s="9">
-        <v>180</v>
-      </c>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B28" s="1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C28" s="2">
         <f>3*60+5</f>
@@ -4462,10 +4107,15 @@
         <f>26+60+(47-14)</f>
         <v>119</v>
       </c>
+      <c r="G28" s="2">
+        <f>(3*60)-(27-14)</f>
+        <v>167</v>
+      </c>
+      <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B29" s="1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C29" s="2">
         <v>72971</v>
@@ -4479,10 +4129,14 @@
       <c r="F29" s="2">
         <v>56245</v>
       </c>
+      <c r="G29" s="2">
+        <v>79365</v>
+      </c>
+      <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B30" s="1" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="C30" s="5">
         <f>C29/C28</f>
@@ -4500,6 +4154,11 @@
         <f>F29/F28</f>
         <v>472.64705882352939</v>
       </c>
+      <c r="G30" s="5">
+        <f>G29/G28</f>
+        <v>475.23952095808386</v>
+      </c>
+      <c r="H30" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added test 6 Freestyle and updated summary
</commit_message>
<xml_diff>
--- a/latest/Spike-SysML Summary.xlsx
+++ b/latest/Spike-SysML Summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jarret\Documents\GitHub\Spike-SysML\development\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FDF0408-A518-447B-82E3-B77BDFA882C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43337E8-06BE-4B90-B739-B660C76C6BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34452" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Cal Runs</t>
   </si>
@@ -51,12 +51,6 @@
   </si>
   <si>
     <t>Verif Runs</t>
-  </si>
-  <si>
-    <t>Op Min Dist</t>
-  </si>
-  <si>
-    <t>Op Max Dist</t>
   </si>
   <si>
     <t>Op Avg Dist</t>
@@ -106,6 +100,19 @@
   <si>
     <t>6 SE</t>
   </si>
+  <si>
+    <t>6 Freestyle</t>
+  </si>
+  <si>
+    <t>Diff</t>
+  </si>
+  <si>
+    <t>Char
+Method</t>
+  </si>
+  <si>
+    <t>Same</t>
+  </si>
 </sst>
 </file>
 
@@ -142,7 +149,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -159,11 +166,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -193,6 +211,22 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -258,7 +292,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$5:$B$8</c:f>
+              <c:f>Sheet1!$B$6:$B$9</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -278,7 +312,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$5:$D$8</c:f>
+              <c:f>Sheet1!$D$6:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -331,7 +365,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$5:$B$8</c:f>
+              <c:f>Sheet1!$B$6:$B$9</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -351,7 +385,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$5:$F$8</c:f>
+              <c:f>Sheet1!$F$6:$F$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -377,8 +411,59 @@
           </c:extLst>
         </c:ser>
         <c:ser>
+          <c:idx val="5"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$H$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$H$6:$H$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-D26B-4A97-922B-37E9C56CEB5E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
           <c:idx val="0"/>
-          <c:order val="2"/>
+          <c:order val="3"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$C$2</c:f>
@@ -402,7 +487,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$5:$B$8</c:f>
+              <c:f>Sheet1!$B$6:$B$9</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -422,7 +507,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$5:$C$8</c:f>
+              <c:f>Sheet1!$C$6:$C$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -449,7 +534,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
-          <c:order val="3"/>
+          <c:order val="4"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$E$2</c:f>
@@ -473,7 +558,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$5:$B$8</c:f>
+              <c:f>Sheet1!$B$6:$B$9</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -493,7 +578,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$8</c:f>
+              <c:f>Sheet1!$E$6:$E$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -520,7 +605,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="4"/>
-          <c:order val="4"/>
+          <c:order val="5"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$G$2</c:f>
@@ -546,7 +631,7 @@
           <c:invertIfNegative val="0"/>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$5:$G$8</c:f>
+              <c:f>Sheet1!$G$6:$G$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -747,10 +832,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -824,11 +906,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$B$9:$B$15</c15:sqref>
+                    <c15:sqref>Sheet1!$B$10:$B$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$11:$B$13,Sheet1!$B$15)</c:f>
+              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -851,11 +933,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$D$9:$D$15</c15:sqref>
+                    <c15:sqref>Sheet1!$D$10:$D$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$D$11:$D$13,Sheet1!$D$15)</c:f>
+              <c:f>(Sheet1!$D$10:$D$12,Sheet1!$D$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
@@ -911,11 +993,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$B$9:$B$15</c15:sqref>
+                    <c15:sqref>Sheet1!$B$10:$B$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$11:$B$13,Sheet1!$B$15)</c:f>
+              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -938,11 +1020,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$F$9:$F$15</c15:sqref>
+                    <c15:sqref>Sheet1!$F$10:$F$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$F$11:$F$13,Sheet1!$F$15)</c:f>
+              <c:f>(Sheet1!$F$10:$F$12,Sheet1!$F$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
@@ -968,8 +1050,88 @@
           </c:extLst>
         </c:ser>
         <c:ser>
+          <c:idx val="5"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$H$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="C00000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="4"/>
+              <c:pt idx="0">
+                <c:v>Op Avg Dist</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Max-Min</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Sdev</c:v>
+              </c:pt>
+              <c:pt idx="3">
+                <c:v>Error</c:v>
+              </c:pt>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:autoCat val="1"/>
+                </c:ext>
+              </c:extLst>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet1!$H$10:$H$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Sheet1!$H$10:$H$12,Sheet1!$H$14)</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>167.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>223</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>101.07145986874831</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>123.4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9C30-4449-AD10-4F9F617C74C0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
           <c:idx val="0"/>
-          <c:order val="2"/>
+          <c:order val="3"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$C$2</c:f>
@@ -996,11 +1158,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$B$9:$B$15</c15:sqref>
+                    <c15:sqref>Sheet1!$B$10:$B$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$11:$B$13,Sheet1!$B$15)</c:f>
+              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1023,11 +1185,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$C$9:$C$15</c15:sqref>
+                    <c15:sqref>Sheet1!$C$10:$C$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$C$11:$C$13,Sheet1!$C$15)</c:f>
+              <c:f>(Sheet1!$C$10:$C$12,Sheet1!$C$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1054,7 +1216,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
-          <c:order val="3"/>
+          <c:order val="4"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$E$2</c:f>
@@ -1081,11 +1243,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$B$9:$B$15</c15:sqref>
+                    <c15:sqref>Sheet1!$B$10:$B$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$11:$B$13,Sheet1!$B$15)</c:f>
+              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1108,11 +1270,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$E$9:$E$15</c15:sqref>
+                    <c15:sqref>Sheet1!$E$10:$E$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$E$11:$E$13,Sheet1!$E$15)</c:f>
+              <c:f>(Sheet1!$E$10:$E$12,Sheet1!$E$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1139,7 +1301,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="4"/>
-          <c:order val="4"/>
+          <c:order val="5"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$G$2</c:f>
@@ -1190,11 +1352,11 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>Sheet1!$G$9:$G$15</c15:sqref>
+                    <c15:sqref>Sheet1!$G$10:$G$14</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$G$11:$G$13,Sheet1!$G$15)</c:f>
+              <c:f>(Sheet1!$G$10:$G$12,Sheet1!$G$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1395,10 +1557,7 @@
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -1468,53 +1627,53 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$16:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$16:$C$27</c:f>
+              <c:f>Sheet1!$C$15:$C$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
-                <c:pt idx="0">
+                <c:ptCount val="13"/>
+                <c:pt idx="1">
                   <c:v>314</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>359</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>641</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>409</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>366</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>469</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>173</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>197</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>171</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>198</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>196</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>200</c:v>
                 </c:pt>
               </c:numCache>
@@ -1556,47 +1715,47 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$16:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$16:$E$25</c:f>
+              <c:f>Sheet1!$E$15:$E$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
+                <c:ptCount val="13"/>
+                <c:pt idx="1">
                   <c:v>442</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>689</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>479</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>264</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>74</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>72</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>71</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>62</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>72</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>77</c:v>
                 </c:pt>
               </c:numCache>
@@ -1635,12 +1794,21 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$B$15:$B$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$16:$G$27</c:f>
+              <c:f>Sheet1!$G$15:$G$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>533</c:v>
                 </c:pt>
@@ -1681,9 +1849,251 @@
             </c:ext>
           </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1430609439"/>
+        <c:axId val="1430609919"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1430609439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1430609919"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:tickMarkSkip val="1"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1430609919"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="900"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Distance</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> to wall (mm)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1430609439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="1"/>
-          <c:order val="3"/>
+          <c:order val="0"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$D$2</c:f>
@@ -1709,41 +2119,41 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$16:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="12"/>
+                <c:ptCount val="13"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$16:$D$23</c:f>
+              <c:f>Sheet1!$D$15:$D$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="8"/>
-                <c:pt idx="0">
+                <c:ptCount val="13"/>
+                <c:pt idx="4">
                   <c:v>395</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="5">
                   <c:v>33</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="6">
                   <c:v>38</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="7">
                   <c:v>99</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="8">
                   <c:v>87</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="9">
                   <c:v>95</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="10">
                   <c:v>81</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="11">
                   <c:v>97</c:v>
                 </c:pt>
               </c:numCache>
@@ -1752,13 +2162,13 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-8D7E-4F84-BBD3-152429E7606B}"/>
+              <c16:uniqueId val="{00000003-0C2B-40B6-B485-71563122C2ED}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="3"/>
-          <c:order val="4"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$F$2</c:f>
@@ -1784,40 +2194,49 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$B$15:$B$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$16:$F$25</c:f>
+              <c:f>Sheet1!$F$15:$F$27</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="10"/>
-                <c:pt idx="0">
+                <c:ptCount val="13"/>
+                <c:pt idx="1">
                   <c:v>228</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>78</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>191</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>178</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>201</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>193</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>257</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>183</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>256</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>180</c:v>
                 </c:pt>
               </c:numCache>
@@ -1826,7 +2245,74 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-8D7E-4F84-BBD3-152429E7606B}"/>
+              <c16:uniqueId val="{00000004-0C2B-40B6-B485-71563122C2ED}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$H$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$H$15:$H$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="2">
+                  <c:v>421</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>224</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>809</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>239</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>248</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>262</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-0C2B-40B6-B485-71563122C2ED}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3141,16 +3627,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>53788</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>134470</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3177,16 +3663,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>55694</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>134471</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>-1</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3215,16 +3701,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
+      <xdr:col>17</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>5</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>516703</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>179293</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3246,6 +3732,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4ECA2C64-86AC-471E-8FDD-2F11C099BDB9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3571,7 +4095,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22FC483D-A2EB-4AB5-93A8-361DFBAB7337}">
-  <dimension ref="B2:H30"/>
+  <dimension ref="B2:I30"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.3984375" customWidth="1"/>
@@ -3580,34 +4104,37 @@
     <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.33203125" customWidth="1"/>
-    <col min="8" max="8" width="2.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="2.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="9.33203125" customWidth="1"/>
+    <col min="9" max="9" width="2.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="2.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C3" s="11">
         <v>46199</v>
@@ -3624,278 +4151,302 @@
       <c r="G3" s="11">
         <v>46203</v>
       </c>
-      <c r="H3" s="10"/>
+      <c r="H3" s="11">
+        <v>46204</v>
+      </c>
+      <c r="I3" s="10"/>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:9" s="17" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="16"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C5" s="3">
         <v>8</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D5" s="3">
         <v>8</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E5" s="3">
         <v>4</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F5" s="3">
         <v>6</v>
-      </c>
-      <c r="G4" s="3">
-        <v>3</v>
-      </c>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B5" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3">
-        <v>0</v>
       </c>
       <c r="G5" s="3">
         <v>3</v>
       </c>
-      <c r="H5" s="3"/>
+      <c r="H5" s="3">
+        <v>6</v>
+      </c>
+      <c r="I5" s="3"/>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3">
         <v>2</v>
       </c>
-      <c r="C6" s="3">
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3">
         <v>1</v>
-      </c>
-      <c r="D6" s="3">
-        <v>4</v>
-      </c>
-      <c r="E6" s="3">
-        <v>0</v>
       </c>
       <c r="F6" s="3">
         <v>0</v>
       </c>
       <c r="G6" s="3">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3"/>
+        <v>3</v>
+      </c>
+      <c r="H6" s="3">
+        <v>1</v>
+      </c>
+      <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B7" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
       </c>
       <c r="D7" s="3">
+        <v>4</v>
+      </c>
+      <c r="E7" s="3">
         <v>0</v>
-      </c>
-      <c r="E7" s="3">
-        <v>2</v>
       </c>
       <c r="F7" s="3">
         <v>0</v>
       </c>
       <c r="G7" s="3">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3">
         <v>2</v>
       </c>
-      <c r="H7" s="3"/>
+      <c r="F8" s="3">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3">
+        <v>2</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3"/>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B8" s="1" t="s">
+    <row r="9" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="7">
+        <f>C8+C5</f>
+        <v>9</v>
+      </c>
+      <c r="D9" s="7">
+        <f>D8+D5</f>
+        <v>8</v>
+      </c>
+      <c r="E9" s="7">
+        <f>E8+E5</f>
+        <v>6</v>
+      </c>
+      <c r="F9" s="7">
+        <f>F8+F5</f>
+        <v>6</v>
+      </c>
+      <c r="G9" s="7">
+        <f>G8+G5</f>
+        <v>5</v>
+      </c>
+      <c r="H9" s="7">
+        <f>H8+H5</f>
+        <v>6</v>
+      </c>
+      <c r="I9" s="3"/>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4">
+        <v>192.4</v>
+      </c>
+      <c r="D10" s="4">
+        <v>91.8</v>
+      </c>
+      <c r="E10" s="4">
+        <v>70.8</v>
+      </c>
+      <c r="F10" s="4">
+        <v>213.8</v>
+      </c>
+      <c r="G10" s="4">
+        <v>148</v>
+      </c>
+      <c r="H10" s="4">
+        <v>167.4</v>
+      </c>
+      <c r="I10" s="4"/>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="5">
+        <v>29</v>
+      </c>
+      <c r="D11" s="5">
+        <v>18</v>
+      </c>
+      <c r="E11" s="5">
+        <v>15</v>
+      </c>
+      <c r="F11" s="5">
+        <v>77</v>
+      </c>
+      <c r="G11" s="5">
+        <v>22</v>
+      </c>
+      <c r="H11" s="5">
+        <v>223</v>
+      </c>
+      <c r="I11" s="5"/>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B12" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="9">
+        <v>10.781465577554844</v>
+      </c>
+      <c r="D12" s="9">
+        <v>6.7646138101151054</v>
+      </c>
+      <c r="E12" s="9">
+        <v>4.8744230427815767</v>
+      </c>
+      <c r="F12" s="9">
+        <v>35.130613430454076</v>
+      </c>
+      <c r="G12" s="9">
+        <v>8.0498447189992426</v>
+      </c>
+      <c r="H12" s="9">
+        <v>101.07145986874831</v>
+      </c>
+      <c r="I12" s="5"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="7">
-        <f>C7+C4</f>
-        <v>9</v>
-      </c>
-      <c r="D8" s="7">
-        <f>D7+D4</f>
-        <v>8</v>
-      </c>
-      <c r="E8" s="7">
-        <f>E7+E4</f>
-        <v>6</v>
-      </c>
-      <c r="F8" s="7">
-        <f>F7+F4</f>
-        <v>6</v>
-      </c>
-      <c r="G8" s="7">
-        <f>G7+G4</f>
-        <v>5</v>
-      </c>
-      <c r="H8" s="3"/>
+      <c r="C13" s="5">
+        <v>189</v>
+      </c>
+      <c r="D13" s="5">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="E13" s="5">
+        <v>78</v>
+      </c>
+      <c r="F13" s="5">
+        <v>55</v>
+      </c>
+      <c r="G13" s="5">
+        <v>44</v>
+      </c>
+      <c r="H13" s="5">
+        <f>AVERAGE(44, 43, 44, 44, 45)</f>
+        <v>44</v>
+      </c>
+      <c r="I13" s="5"/>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C9" s="4">
-        <v>171</v>
-      </c>
-      <c r="D9" s="4">
-        <v>81</v>
-      </c>
-      <c r="E9" s="4">
-        <v>62</v>
-      </c>
-      <c r="F9" s="4">
-        <v>180</v>
-      </c>
-      <c r="G9" s="4">
-        <v>135</v>
-      </c>
-      <c r="H9" s="4"/>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="9">
+        <f>C10-C13</f>
+        <v>3.4000000000000057</v>
+      </c>
+      <c r="D14" s="9">
+        <f>D10-D13</f>
+        <v>26.399999999999991</v>
+      </c>
+      <c r="E14" s="9">
+        <f>E10-E13</f>
+        <v>-7.2000000000000028</v>
+      </c>
+      <c r="F14" s="9">
+        <f>F10-F13</f>
+        <v>158.80000000000001</v>
+      </c>
+      <c r="G14" s="9">
+        <f>G10-G13</f>
+        <v>104</v>
+      </c>
+      <c r="H14" s="9">
+        <f>H10-H13</f>
+        <v>123.4</v>
+      </c>
+      <c r="I14" s="5"/>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="4">
-        <v>200</v>
-      </c>
-      <c r="D10" s="4">
-        <v>99</v>
-      </c>
-      <c r="E10" s="4">
-        <v>77</v>
-      </c>
-      <c r="F10" s="4">
-        <v>257</v>
-      </c>
-      <c r="G10" s="4">
-        <v>157</v>
-      </c>
-      <c r="H10" s="4"/>
+    <row r="15" spans="2:9" x14ac:dyDescent="0.45">
+      <c r="B15" s="1"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="3">
+        <v>533</v>
+      </c>
+      <c r="H15" s="3"/>
+      <c r="I15" s="2"/>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="4">
-        <v>192.4</v>
-      </c>
-      <c r="D11" s="4">
-        <v>91.8</v>
-      </c>
-      <c r="E11" s="4">
-        <v>70.8</v>
-      </c>
-      <c r="F11" s="4">
-        <v>213.8</v>
-      </c>
-      <c r="G11" s="4">
-        <v>148</v>
-      </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="5">
-        <v>29</v>
-      </c>
-      <c r="D12" s="5">
-        <v>18</v>
-      </c>
-      <c r="E12" s="5">
-        <v>15</v>
-      </c>
-      <c r="F12" s="5">
-        <v>77</v>
-      </c>
-      <c r="G12" s="5">
-        <v>22</v>
-      </c>
-      <c r="H12" s="5"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C13" s="9">
-        <v>10.781465577554844</v>
-      </c>
-      <c r="D13" s="9">
-        <v>6.7646138101151054</v>
-      </c>
-      <c r="E13" s="9">
-        <v>4.8744230427815767</v>
-      </c>
-      <c r="F13" s="9">
-        <v>35.130613430454076</v>
-      </c>
-      <c r="G13" s="9">
-        <v>8.0498447189992426</v>
-      </c>
-      <c r="H13" s="5"/>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="5">
-        <v>189</v>
-      </c>
-      <c r="D14" s="5">
-        <v>65.400000000000006</v>
-      </c>
-      <c r="E14" s="5">
-        <v>78</v>
-      </c>
-      <c r="F14" s="5">
-        <v>55</v>
-      </c>
-      <c r="G14" s="5">
-        <v>44</v>
-      </c>
-      <c r="H14" s="5"/>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="9">
-        <f>C11-C14</f>
-        <v>3.4000000000000057</v>
-      </c>
-      <c r="D15" s="9">
-        <f>D11-D14</f>
-        <v>26.399999999999991</v>
-      </c>
-      <c r="E15" s="9">
-        <f>E11-E14</f>
-        <v>-7.2000000000000028</v>
-      </c>
-      <c r="F15" s="9">
-        <f>F11-F14</f>
-        <v>158.80000000000001</v>
-      </c>
-      <c r="G15" s="9">
-        <f>G11-G14</f>
-        <v>104</v>
-      </c>
-      <c r="H15" s="5"/>
-    </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B16" s="1"/>
       <c r="C16" s="2">
         <v>314</v>
       </c>
-      <c r="D16" s="2">
-        <v>395</v>
-      </c>
+      <c r="D16" s="2"/>
       <c r="E16" s="2">
         <v>442</v>
       </c>
@@ -3903,18 +4454,17 @@
         <v>228</v>
       </c>
       <c r="G16" s="3">
-        <v>533</v>
-      </c>
-      <c r="H16" s="2"/>
+        <v>498</v>
+      </c>
+      <c r="H16" s="3"/>
+      <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B17" s="1"/>
       <c r="C17" s="2">
         <v>359</v>
       </c>
-      <c r="D17" s="2">
-        <v>33</v>
-      </c>
+      <c r="D17" s="2"/>
       <c r="E17" s="2">
         <v>689</v>
       </c>
@@ -3922,18 +4472,19 @@
         <v>78</v>
       </c>
       <c r="G17" s="3">
-        <v>498</v>
-      </c>
-      <c r="H17" s="2"/>
+        <v>530</v>
+      </c>
+      <c r="H17" s="2">
+        <v>421</v>
+      </c>
+      <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B18" s="1"/>
       <c r="C18" s="2">
         <v>641</v>
       </c>
-      <c r="D18" s="2">
-        <v>38</v>
-      </c>
+      <c r="D18" s="2"/>
       <c r="E18" s="2">
         <v>479</v>
       </c>
@@ -3941,17 +4492,20 @@
         <v>191</v>
       </c>
       <c r="G18" s="3">
-        <v>530</v>
-      </c>
-      <c r="H18" s="2"/>
+        <v>138</v>
+      </c>
+      <c r="H18" s="2">
+        <v>224</v>
+      </c>
+      <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B19" s="1"/>
       <c r="C19" s="2">
         <v>409</v>
       </c>
       <c r="D19" s="2">
-        <v>99</v>
+        <v>395</v>
       </c>
       <c r="E19" s="2">
         <v>264</v>
@@ -3960,17 +4514,19 @@
         <v>178</v>
       </c>
       <c r="G19" s="3">
-        <v>138</v>
-      </c>
-      <c r="H19" s="2"/>
+        <v>148</v>
+      </c>
+      <c r="H19" s="2">
+        <v>809</v>
+      </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B20" s="1"/>
       <c r="C20" s="2">
         <v>366</v>
       </c>
       <c r="D20" s="2">
-        <v>87</v>
+        <v>33</v>
       </c>
       <c r="E20" s="2">
         <v>74</v>
@@ -3979,16 +4535,19 @@
         <v>201</v>
       </c>
       <c r="G20" s="3">
-        <v>148</v>
+        <v>157</v>
+      </c>
+      <c r="H20" s="2">
+        <v>129</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B21" s="1"/>
       <c r="C21" s="2">
         <v>469</v>
       </c>
       <c r="D21" s="2">
-        <v>95</v>
+        <v>38</v>
       </c>
       <c r="E21" s="2">
         <v>72</v>
@@ -3997,16 +4556,19 @@
         <v>193</v>
       </c>
       <c r="G21" s="3">
-        <v>157</v>
+        <v>135</v>
+      </c>
+      <c r="H21" s="2">
+        <v>39</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B22" s="1"/>
       <c r="C22" s="2">
         <v>173</v>
       </c>
       <c r="D22" s="2">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="E22" s="2">
         <v>71</v>
@@ -4015,16 +4577,20 @@
         <v>257</v>
       </c>
       <c r="G22" s="3">
-        <v>135</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="H22" s="2">
+        <v>49</v>
+      </c>
+      <c r="I22" s="2"/>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B23" s="1"/>
       <c r="C23" s="2">
         <v>197</v>
       </c>
       <c r="D23" s="2">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E23" s="2">
         <v>62</v>
@@ -4033,15 +4599,21 @@
         <v>183</v>
       </c>
       <c r="G23" s="3">
-        <v>145</v>
-      </c>
-      <c r="H23" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="H23" s="2">
+        <v>239</v>
+      </c>
+      <c r="I23" s="2"/>
     </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B24" s="1"/>
       <c r="C24" s="2">
         <v>171</v>
       </c>
+      <c r="D24" s="2">
+        <v>95</v>
+      </c>
       <c r="E24" s="2">
         <v>72</v>
       </c>
@@ -4049,47 +4621,60 @@
         <v>256</v>
       </c>
       <c r="G24" s="3">
-        <v>147</v>
-      </c>
-      <c r="H24" s="2"/>
+        <v>156</v>
+      </c>
+      <c r="H24" s="2">
+        <v>248</v>
+      </c>
+      <c r="I24" s="2"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B25" s="1"/>
       <c r="C25" s="2">
         <v>198</v>
       </c>
+      <c r="D25" s="2">
+        <v>81</v>
+      </c>
       <c r="E25" s="2">
         <v>77</v>
       </c>
       <c r="F25" s="2">
         <v>180</v>
       </c>
-      <c r="G25" s="3">
-        <v>156</v>
-      </c>
-      <c r="H25" s="2"/>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2">
+        <v>262</v>
+      </c>
+      <c r="I25" s="2"/>
     </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B26" s="1"/>
-      <c r="C26" s="2">
+      <c r="C26" s="13">
         <v>196</v>
       </c>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
+      <c r="D26" s="13">
+        <v>97</v>
+      </c>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
     </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B27" s="1"/>
       <c r="C27" s="6">
         <v>200</v>
       </c>
-      <c r="D27" s="8"/>
+      <c r="D27" s="6"/>
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
       <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B28" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C28" s="2">
         <f>3*60+5</f>
@@ -4112,10 +4697,11 @@
         <v>167</v>
       </c>
       <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B29" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C29" s="2">
         <v>72971</v>
@@ -4133,10 +4719,11 @@
         <v>79365</v>
       </c>
       <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B30" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C30" s="5">
         <f>C29/C28</f>
@@ -4159,6 +4746,7 @@
         <v>475.23952095808386</v>
       </c>
       <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added test 7 and updated summary.
</commit_message>
<xml_diff>
--- a/latest/Spike-SysML Summary.xlsx
+++ b/latest/Spike-SysML Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jarret\Documents\GitHub\Spike-SysML\development\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43337E8-06BE-4B90-B739-B660C76C6BA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2E98B0-BC68-442F-A9D4-621C25F43E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34452" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,27 +39,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="27">
   <si>
     <t>Cal Runs</t>
-  </si>
-  <si>
-    <t>Interventions</t>
-  </si>
-  <si>
-    <t>Impacts</t>
   </si>
   <si>
     <t>Verif Runs</t>
   </si>
   <si>
     <t>Op Avg Dist</t>
-  </si>
-  <si>
-    <t>Max-Min</t>
-  </si>
-  <si>
-    <t>Sdev</t>
   </si>
   <si>
     <t>Test</t>
@@ -95,9 +83,6 @@
     <t>Predicted</t>
   </si>
   <si>
-    <t>Error</t>
-  </si>
-  <si>
     <t>6 SE</t>
   </si>
   <si>
@@ -107,11 +92,36 @@
     <t>Diff</t>
   </si>
   <si>
-    <t>Char
+    <t>Same</t>
+  </si>
+  <si>
+    <t>7 SE</t>
+  </si>
+  <si>
+    <t>v1 Char
 Method</t>
   </si>
   <si>
-    <t>Same</t>
+    <t>v0</t>
+  </si>
+  <si>
+    <t>v2 Sens
+Anomoly</t>
+  </si>
+  <si>
+    <t>Op Max-Min</t>
+  </si>
+  <si>
+    <t>Op Error</t>
+  </si>
+  <si>
+    <t>Op Sdev</t>
+  </si>
+  <si>
+    <t>Char Int</t>
+  </si>
+  <si>
+    <t>Char Imp</t>
   </si>
 </sst>
 </file>
@@ -181,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -210,10 +220,6 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -296,10 +302,10 @@
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Interventions</c:v>
+                  <c:v>Char Int</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Impacts</c:v>
+                  <c:v>Char Imp</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Verif Runs</c:v>
@@ -369,10 +375,10 @@
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Interventions</c:v>
+                  <c:v>Char Int</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Impacts</c:v>
+                  <c:v>Char Imp</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Verif Runs</c:v>
@@ -491,10 +497,10 @@
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Interventions</c:v>
+                  <c:v>Char Int</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Impacts</c:v>
+                  <c:v>Char Imp</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Verif Runs</c:v>
@@ -562,10 +568,10 @@
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>Interventions</c:v>
+                  <c:v>Char Int</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Impacts</c:v>
+                  <c:v>Char Imp</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>Verif Runs</c:v>
@@ -653,6 +659,59 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-1C6B-4A7D-8E9A-CBC3F1217CFE}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$I$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$I$6:$I$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5DE2-49A7-8D50-2EEB127B1C03}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -910,20 +969,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
+              <c:f>(Sheet1!$B$10,Sheet1!$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>Op Avg Dist</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Max-Min</c:v>
+                  <c:v>Op Sdev</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sdev</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Error</c:v>
+                  <c:v>Op Error</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -937,20 +993,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$D$10:$D$12,Sheet1!$D$14)</c:f>
+              <c:f>(Sheet1!$D$10,Sheet1!$D$12,Sheet1!$D$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>91.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>18</c:v>
+                  <c:v>6.7646138101151054</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.7646138101151054</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>26.399999999999991</c:v>
                 </c:pt>
               </c:numCache>
@@ -997,20 +1050,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
+              <c:f>(Sheet1!$B$10,Sheet1!$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>Op Avg Dist</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Max-Min</c:v>
+                  <c:v>Op Sdev</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sdev</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Error</c:v>
+                  <c:v>Op Error</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1024,20 +1074,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$F$10:$F$12,Sheet1!$F$14)</c:f>
+              <c:f>(Sheet1!$F$10,Sheet1!$F$12,Sheet1!$F$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>213.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>77</c:v>
+                  <c:v>35.130613430454076</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>35.130613430454076</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>158.80000000000001</c:v>
                 </c:pt>
               </c:numCache>
@@ -1075,18 +1122,15 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="4"/>
+              <c:ptCount val="3"/>
               <c:pt idx="0">
                 <c:v>Op Avg Dist</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>Max-Min</c:v>
+                <c:v>Op Sdev</c:v>
               </c:pt>
               <c:pt idx="2">
-                <c:v>Sdev</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>Error</c:v>
+                <c:v>Op Error</c:v>
               </c:pt>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
@@ -1104,20 +1148,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$H$10:$H$12,Sheet1!$H$14)</c:f>
+              <c:f>(Sheet1!$H$10,Sheet1!$H$12,Sheet1!$H$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>167.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>223</c:v>
+                  <c:v>101.07145986874831</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>101.07145986874831</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>123.4</c:v>
                 </c:pt>
               </c:numCache>
@@ -1162,20 +1203,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
+              <c:f>(Sheet1!$B$10,Sheet1!$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>Op Avg Dist</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Max-Min</c:v>
+                  <c:v>Op Sdev</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sdev</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Error</c:v>
+                  <c:v>Op Error</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1189,20 +1227,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$C$10:$C$12,Sheet1!$C$14)</c:f>
+              <c:f>(Sheet1!$C$10,Sheet1!$C$12,Sheet1!$C$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>192.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>29</c:v>
+                  <c:v>10.781465577554844</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10.781465577554844</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>3.4000000000000057</c:v>
                 </c:pt>
               </c:numCache>
@@ -1247,20 +1282,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$B$10:$B$12,Sheet1!$B$14)</c:f>
+              <c:f>(Sheet1!$B$10,Sheet1!$B$12,Sheet1!$B$14)</c:f>
               <c:strCache>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>Op Avg Dist</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Max-Min</c:v>
+                  <c:v>Op Sdev</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Sdev</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Error</c:v>
+                  <c:v>Op Error</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1274,20 +1306,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$E$10:$E$12,Sheet1!$E$14)</c:f>
+              <c:f>(Sheet1!$E$10,Sheet1!$E$12,Sheet1!$E$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>70.8</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15</c:v>
+                  <c:v>4.8744230427815767</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4.8744230427815767</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>-7.2000000000000028</c:v>
                 </c:pt>
               </c:numCache>
@@ -1327,18 +1356,15 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strLit>
-              <c:ptCount val="4"/>
+              <c:ptCount val="3"/>
               <c:pt idx="0">
                 <c:v>Op Avg Dist</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>Max-Min</c:v>
+                <c:v>Op Sdev</c:v>
               </c:pt>
               <c:pt idx="2">
-                <c:v>Sdev</c:v>
-              </c:pt>
-              <c:pt idx="3">
-                <c:v>Error</c:v>
+                <c:v>Op Error</c:v>
               </c:pt>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
@@ -1356,20 +1382,17 @@
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>(Sheet1!$G$10:$G$12,Sheet1!$G$14)</c:f>
+              <c:f>(Sheet1!$G$10,Sheet1!$G$12,Sheet1!$G$14)</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>148</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>22</c:v>
+                  <c:v>8.0498447189992426</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8.0498447189992426</c:v>
-                </c:pt>
-                <c:pt idx="3">
                   <c:v>104</c:v>
                 </c:pt>
               </c:numCache>
@@ -1378,6 +1401,82 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-D6E6-4A6C-8AC9-E6D23C79F65F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$I$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>Op Avg Dist</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Op Sdev</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Op Error</c:v>
+              </c:pt>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:autoCat val="1"/>
+                </c:ext>
+              </c:extLst>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet1!$I$10:$I$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Sheet1!$I$10,Sheet1!$I$12,Sheet1!$I$14)</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.3560994328282812</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0EFF-4E63-AAD3-740ADE87300B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1627,53 +1726,53 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$15:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$15:$C$27</c:f>
+              <c:f>Sheet1!$C$15:$C$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
-                <c:pt idx="1">
+                <c:ptCount val="14"/>
+                <c:pt idx="2">
                   <c:v>314</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>359</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>641</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>409</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>366</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>469</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>173</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>197</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>171</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>198</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>196</c:v>
                 </c:pt>
-                <c:pt idx="12">
+                <c:pt idx="13">
                   <c:v>200</c:v>
                 </c:pt>
               </c:numCache>
@@ -1715,19 +1814,19 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$15:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$15:$E$27</c:f>
+              <c:f>Sheet1!$E$15:$E$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="1">
                   <c:v>442</c:v>
                 </c:pt>
@@ -1796,19 +1895,19 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$15:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$15:$G$27</c:f>
+              <c:f>Sheet1!$G$15:$G$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>533</c:v>
                 </c:pt>
@@ -1846,6 +1945,78 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{0000000B-8D7E-4F84-BBD3-152429E7606B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$I$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$I$15:$I$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="1">
+                  <c:v>196</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>138</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6C96-4787-83E0-51DC73D3E7C2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2092,7 +2263,7 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="1"/>
+          <c:idx val="3"/>
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
@@ -2119,41 +2290,41 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$15:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$15:$D$27</c:f>
+              <c:f>Sheet1!$D$15:$D$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
-                <c:pt idx="4">
+                <c:ptCount val="14"/>
+                <c:pt idx="5">
                   <c:v>395</c:v>
                 </c:pt>
-                <c:pt idx="5">
+                <c:pt idx="6">
                   <c:v>33</c:v>
                 </c:pt>
-                <c:pt idx="6">
+                <c:pt idx="7">
                   <c:v>38</c:v>
                 </c:pt>
-                <c:pt idx="7">
+                <c:pt idx="8">
                   <c:v>99</c:v>
                 </c:pt>
-                <c:pt idx="8">
+                <c:pt idx="9">
                   <c:v>87</c:v>
                 </c:pt>
-                <c:pt idx="9">
+                <c:pt idx="10">
                   <c:v>95</c:v>
                 </c:pt>
-                <c:pt idx="10">
+                <c:pt idx="11">
                   <c:v>81</c:v>
                 </c:pt>
-                <c:pt idx="11">
+                <c:pt idx="12">
                   <c:v>97</c:v>
                 </c:pt>
               </c:numCache>
@@ -2162,12 +2333,12 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-0C2B-40B6-B485-71563122C2ED}"/>
+              <c16:uniqueId val="{00000008-7F1F-4544-A3B9-23B6184D29A5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="3"/>
+          <c:idx val="5"/>
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
@@ -2196,19 +2367,19 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$B$15:$B$27</c:f>
+              <c:f>Sheet1!$B$15:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$15:$F$27</c:f>
+              <c:f>Sheet1!$F$15:$F$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="1">
                   <c:v>228</c:v>
                 </c:pt>
@@ -2245,12 +2416,12 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-0C2B-40B6-B485-71563122C2ED}"/>
+              <c16:uniqueId val="{00000009-7F1F-4544-A3B9-23B6184D29A5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="0"/>
+          <c:idx val="6"/>
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
@@ -2273,12 +2444,21 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$B$15:$B$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$15:$H$27</c:f>
+              <c:f>Sheet1!$H$15:$H$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="2">
                   <c:v>421</c:v>
                 </c:pt>
@@ -2312,7 +2492,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-0C2B-40B6-B485-71563122C2ED}"/>
+              <c16:uniqueId val="{0000000A-7F1F-4544-A3B9-23B6184D29A5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2384,6 +2564,7 @@
         <c:axId val="1430609919"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="900"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -3627,7 +3808,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -3663,7 +3844,7 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -3672,7 +3853,7 @@
       <xdr:col>16</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>-1</xdr:rowOff>
+      <xdr:rowOff>179293</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3747,7 +3928,7 @@
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>29</xdr:row>
+      <xdr:row>30</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -4095,7 +4276,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22FC483D-A2EB-4AB5-93A8-361DFBAB7337}">
-  <dimension ref="B2:I30"/>
+  <dimension ref="B2:J31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.3984375" customWidth="1"/>
@@ -4104,37 +4285,40 @@
     <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="9.33203125" customWidth="1"/>
-    <col min="9" max="9" width="2.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="9.33203125" customWidth="1"/>
+    <col min="10" max="10" width="2.33203125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="2.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="G2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="B3" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B3" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C3" s="11">
         <v>46199</v>
@@ -4154,29 +4338,37 @@
       <c r="H3" s="11">
         <v>46204</v>
       </c>
-      <c r="I3" s="10"/>
+      <c r="I3" s="11">
+        <v>46205</v>
+      </c>
+      <c r="J3" s="10"/>
     </row>
-    <row r="4" spans="2:9" s="17" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:10" s="15" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="12"/>
+      <c r="E4" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="16"/>
+      <c r="J4" s="14"/>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
@@ -4198,11 +4390,14 @@
       <c r="H5" s="3">
         <v>6</v>
       </c>
-      <c r="I5" s="3"/>
+      <c r="I5" s="3">
+        <v>4</v>
+      </c>
+      <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B6" s="1" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C6" s="3">
         <v>2</v>
@@ -4222,11 +4417,14 @@
       <c r="H6" s="3">
         <v>1</v>
       </c>
-      <c r="I6" s="3"/>
+      <c r="I6" s="3">
+        <v>4</v>
+      </c>
+      <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B7" s="1" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="C7" s="3">
         <v>1</v>
@@ -4246,11 +4444,14 @@
       <c r="H7" s="3">
         <v>0</v>
       </c>
-      <c r="I7" s="3"/>
+      <c r="I7" s="3">
+        <v>1</v>
+      </c>
+      <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B8" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C8" s="3">
         <v>1</v>
@@ -4270,41 +4471,48 @@
       <c r="H8" s="3">
         <v>0</v>
       </c>
-      <c r="I8" s="3"/>
+      <c r="I8" s="3">
+        <v>2</v>
+      </c>
+      <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C9" s="7">
-        <f>C8+C5</f>
+        <f t="shared" ref="C9:I9" si="0">C8+C5</f>
         <v>9</v>
       </c>
       <c r="D9" s="7">
-        <f>D8+D5</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="E9" s="7">
-        <f>E8+E5</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="F9" s="7">
-        <f>F8+F5</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="G9" s="7">
-        <f>G8+G5</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="H9" s="7">
-        <f>H8+H5</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="I9" s="3"/>
+      <c r="I9" s="7">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B10" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C10" s="4">
         <v>192.4</v>
@@ -4324,11 +4532,14 @@
       <c r="H10" s="4">
         <v>167.4</v>
       </c>
-      <c r="I10" s="4"/>
+      <c r="I10" s="4">
+        <v>44</v>
+      </c>
+      <c r="J10" s="4"/>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B11" s="1" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C11" s="5">
         <v>29</v>
@@ -4348,11 +4559,14 @@
       <c r="H11" s="5">
         <v>223</v>
       </c>
-      <c r="I11" s="5"/>
+      <c r="I11" s="5">
+        <v>19</v>
+      </c>
+      <c r="J11" s="5"/>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B12" s="1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C12" s="9">
         <v>10.781465577554844</v>
@@ -4372,11 +4586,14 @@
       <c r="H12" s="9">
         <v>101.07145986874831</v>
       </c>
-      <c r="I12" s="5"/>
+      <c r="I12" s="9">
+        <v>6.3560994328282812</v>
+      </c>
+      <c r="J12" s="5"/>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B13" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C13" s="5">
         <v>189</v>
@@ -4397,39 +4614,46 @@
         <f>AVERAGE(44, 43, 44, 44, 45)</f>
         <v>44</v>
       </c>
-      <c r="I13" s="5"/>
+      <c r="I13" s="5">
+        <v>55</v>
+      </c>
+      <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B14" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C14" s="9">
-        <f>C10-C13</f>
+        <f t="shared" ref="C14:I14" si="1">C10-C13</f>
         <v>3.4000000000000057</v>
       </c>
       <c r="D14" s="9">
-        <f>D10-D13</f>
+        <f t="shared" si="1"/>
         <v>26.399999999999991</v>
       </c>
       <c r="E14" s="9">
-        <f>E10-E13</f>
+        <f t="shared" si="1"/>
         <v>-7.2000000000000028</v>
       </c>
       <c r="F14" s="9">
-        <f>F10-F13</f>
+        <f t="shared" si="1"/>
         <v>158.80000000000001</v>
       </c>
       <c r="G14" s="9">
-        <f>G10-G13</f>
+        <f t="shared" si="1"/>
         <v>104</v>
       </c>
       <c r="H14" s="9">
-        <f>H10-H13</f>
+        <f t="shared" si="1"/>
         <v>123.4</v>
       </c>
-      <c r="I14" s="5"/>
+      <c r="I14" s="9">
+        <f t="shared" si="1"/>
+        <v>-11</v>
+      </c>
+      <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B15" s="1"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -4439,13 +4663,11 @@
         <v>533</v>
       </c>
       <c r="H15" s="3"/>
-      <c r="I15" s="2"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B16" s="1"/>
-      <c r="C16" s="2">
-        <v>314</v>
-      </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2">
         <v>442</v>
@@ -4457,12 +4679,15 @@
         <v>498</v>
       </c>
       <c r="H16" s="3"/>
-      <c r="I16" s="2"/>
+      <c r="I16" s="2">
+        <v>196</v>
+      </c>
+      <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B17" s="1"/>
       <c r="C17" s="2">
-        <v>359</v>
+        <v>314</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2">
@@ -4477,12 +4702,15 @@
       <c r="H17" s="2">
         <v>421</v>
       </c>
-      <c r="I17" s="2"/>
+      <c r="I17" s="2">
+        <v>113</v>
+      </c>
+      <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B18" s="1"/>
       <c r="C18" s="2">
-        <v>641</v>
+        <v>359</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2">
@@ -4497,16 +4725,17 @@
       <c r="H18" s="2">
         <v>224</v>
       </c>
-      <c r="I18" s="2"/>
+      <c r="I18" s="2">
+        <v>138</v>
+      </c>
+      <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B19" s="1"/>
       <c r="C19" s="2">
-        <v>409</v>
-      </c>
-      <c r="D19" s="2">
-        <v>395</v>
-      </c>
+        <v>641</v>
+      </c>
+      <c r="D19" s="2"/>
       <c r="E19" s="2">
         <v>264</v>
       </c>
@@ -4519,14 +4748,17 @@
       <c r="H19" s="2">
         <v>809</v>
       </c>
+      <c r="I19" s="2">
+        <v>28</v>
+      </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B20" s="1"/>
       <c r="C20" s="2">
-        <v>366</v>
+        <v>409</v>
       </c>
       <c r="D20" s="2">
-        <v>33</v>
+        <v>395</v>
       </c>
       <c r="E20" s="2">
         <v>74</v>
@@ -4540,14 +4772,17 @@
       <c r="H20" s="2">
         <v>129</v>
       </c>
+      <c r="I20" s="2">
+        <v>46</v>
+      </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B21" s="1"/>
       <c r="C21" s="2">
-        <v>469</v>
+        <v>366</v>
       </c>
       <c r="D21" s="2">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E21" s="2">
         <v>72</v>
@@ -4561,14 +4796,17 @@
       <c r="H21" s="2">
         <v>39</v>
       </c>
+      <c r="I21" s="2">
+        <v>46</v>
+      </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B22" s="1"/>
       <c r="C22" s="2">
-        <v>173</v>
+        <v>469</v>
       </c>
       <c r="D22" s="2">
-        <v>99</v>
+        <v>38</v>
       </c>
       <c r="E22" s="2">
         <v>71</v>
@@ -4582,15 +4820,18 @@
       <c r="H22" s="2">
         <v>49</v>
       </c>
-      <c r="I22" s="2"/>
+      <c r="I22" s="2">
+        <v>45</v>
+      </c>
+      <c r="J22" s="2"/>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B23" s="1"/>
       <c r="C23" s="2">
-        <v>197</v>
+        <v>173</v>
       </c>
       <c r="D23" s="2">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="E23" s="2">
         <v>62</v>
@@ -4604,15 +4845,18 @@
       <c r="H23" s="2">
         <v>239</v>
       </c>
-      <c r="I23" s="2"/>
+      <c r="I23" s="2">
+        <v>32</v>
+      </c>
+      <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B24" s="1"/>
       <c r="C24" s="2">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D24" s="2">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E24" s="2">
         <v>72</v>
@@ -4626,15 +4870,18 @@
       <c r="H24" s="2">
         <v>248</v>
       </c>
-      <c r="I24" s="2"/>
+      <c r="I24" s="2">
+        <v>51</v>
+      </c>
+      <c r="J24" s="2"/>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B25" s="1"/>
       <c r="C25" s="2">
-        <v>198</v>
+        <v>171</v>
       </c>
       <c r="D25" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="E25" s="2">
         <v>77</v>
@@ -4646,107 +4893,129 @@
       <c r="H25" s="2">
         <v>262</v>
       </c>
-      <c r="I25" s="2"/>
+      <c r="I25" s="2">
+        <v>46</v>
+      </c>
+      <c r="J25" s="2"/>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B26" s="1"/>
-      <c r="C26" s="13">
+      <c r="C26" s="2">
+        <v>198</v>
+      </c>
+      <c r="D26" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="B27" s="1"/>
+      <c r="C27" s="2">
         <v>196</v>
       </c>
-      <c r="D26" s="13">
+      <c r="D27" s="2">
         <v>97</v>
       </c>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B27" s="1"/>
-      <c r="C27" s="6">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="B28" s="1"/>
+      <c r="C28" s="6">
         <v>200</v>
       </c>
-      <c r="D27" s="6"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B28" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="2">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="B29" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" s="2">
         <f>3*60+5</f>
         <v>185</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D29" s="3">
         <f>(57+52)</f>
         <v>109</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E29" s="3">
         <f>2*60+12</f>
         <v>132</v>
       </c>
-      <c r="F28" s="2">
+      <c r="F29" s="2">
         <f>26+60+(47-14)</f>
         <v>119</v>
       </c>
-      <c r="G28" s="2">
+      <c r="G29" s="2">
         <f>(3*60)-(27-14)</f>
         <v>167</v>
       </c>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
+      <c r="H29" s="2">
+        <f>2*60+16+22</f>
+        <v>158</v>
+      </c>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B29" s="1" t="s">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="B30" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="2">
+        <v>72971</v>
+      </c>
+      <c r="D30" s="3">
+        <v>67098</v>
+      </c>
+      <c r="E30" s="3">
+        <v>61254</v>
+      </c>
+      <c r="F30" s="2">
+        <v>56245</v>
+      </c>
+      <c r="G30" s="2">
+        <v>79365</v>
+      </c>
+      <c r="H30" s="2">
+        <v>46321</v>
+      </c>
+      <c r="I30" s="2">
+        <v>30857</v>
+      </c>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="B31" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C29" s="2">
-        <v>72971</v>
-      </c>
-      <c r="D29" s="3">
-        <v>67098</v>
-      </c>
-      <c r="E29" s="3">
-        <v>61254</v>
-      </c>
-      <c r="F29" s="2">
-        <v>56245</v>
-      </c>
-      <c r="G29" s="2">
-        <v>79365</v>
-      </c>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="B30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="5">
-        <f>C29/C28</f>
+      <c r="C31" s="5">
+        <f t="shared" ref="C31:H31" si="2">C30/C29</f>
         <v>394.43783783783783</v>
       </c>
-      <c r="D30" s="5">
-        <f>D29/D28</f>
+      <c r="D31" s="5">
+        <f t="shared" si="2"/>
         <v>615.57798165137615</v>
       </c>
-      <c r="E30" s="5">
-        <f>E29/E28</f>
+      <c r="E31" s="5">
+        <f t="shared" si="2"/>
         <v>464.04545454545456</v>
       </c>
-      <c r="F30" s="5">
-        <f>F29/F28</f>
+      <c r="F31" s="5">
+        <f t="shared" si="2"/>
         <v>472.64705882352939</v>
       </c>
-      <c r="G30" s="5">
-        <f>G29/G28</f>
+      <c r="G31" s="5">
+        <f t="shared" si="2"/>
         <v>475.23952095808386</v>
       </c>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
+      <c r="H31" s="5">
+        <f t="shared" si="2"/>
+        <v>293.17088607594934</v>
+      </c>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added test 8 SE
</commit_message>
<xml_diff>
--- a/latest/Spike-SysML Summary.xlsx
+++ b/latest/Spike-SysML Summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jarret\Documents\GitHub\Spike-SysML\development\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE1CE244-5471-4F96-BC04-E17F698B68A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C8620C-DA09-48E2-AE1D-60CA2BEFF7D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34452" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
   <si>
     <t>Cal Runs</t>
   </si>
@@ -123,6 +123,9 @@
   <si>
     <t>Impacts</t>
   </si>
+  <si>
+    <t>8 SE</t>
+  </si>
 </sst>
 </file>
 
@@ -191,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -237,6 +240,26 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -773,6 +796,57 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-5DE2-49A7-8D50-2EEB127B1C03}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="8"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="tx2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$K$6:$K$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-AA23-4BCE-B4AA-96F5375311F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1146,7 +1220,7 @@
                   <c:v>39.277219860881154</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>158.80000000000001</c:v>
+                  <c:v>154.80000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1296,7 +1370,7 @@
                   <c:v>13.049904214207857</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>133.4</c:v>
+                  <c:v>130.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1614,6 +1688,80 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-0EFF-4E63-AAD3-740ADE87300B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="8"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="tx2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strLit>
+              <c:ptCount val="3"/>
+              <c:pt idx="0">
+                <c:v>Op Avg Dist</c:v>
+              </c:pt>
+              <c:pt idx="1">
+                <c:v>Op Sdev</c:v>
+              </c:pt>
+              <c:pt idx="2">
+                <c:v>Op Error</c:v>
+              </c:pt>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:autoCat val="1"/>
+                </c:ext>
+              </c:extLst>
+            </c:strLit>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                  <c15:fullRef>
+                    <c15:sqref>Sheet1!$K$10:$K$14</c15:sqref>
+                  </c15:fullRef>
+                </c:ext>
+              </c:extLst>
+              <c:f>(Sheet1!$K$10,Sheet1!$K$12,Sheet1!$K$14)</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>43.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7.700649323271394</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>-1.6000000000000014</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A58A-4008-B98F-40A74B0C5393}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1863,7 +2011,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$15:$B$28</c:f>
+              <c:f>Sheet1!$B$16:$B$29</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1874,7 +2022,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$15:$C$28</c:f>
+              <c:f>Sheet1!$C$16:$C$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -1953,7 +2101,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$15:$B$28</c:f>
+              <c:f>Sheet1!$B$16:$B$29</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1964,7 +2112,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$15:$E$28</c:f>
+              <c:f>Sheet1!$E$16:$E$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -2036,7 +2184,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$15:$B$28</c:f>
+              <c:f>Sheet1!$B$16:$B$29</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2047,7 +2195,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$15:$G$28</c:f>
+              <c:f>Sheet1!$G$16:$G$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -2119,7 +2267,7 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$15:$I$28</c:f>
+              <c:f>Sheet1!$I$16:$I$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -2160,6 +2308,76 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-6C96-4787-83E0-51DC73D3E7C2}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$K$16:$K$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>515</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>522</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>513</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>542</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>48</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-83A0-4E10-8A4A-E849A2DB9629}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2433,7 +2651,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$15:$B$28</c:f>
+              <c:f>Sheet1!$B$16:$B$29</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2444,7 +2662,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$15:$D$28</c:f>
+              <c:f>Sheet1!$D$16:$D$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -2512,7 +2730,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$15:$B$28</c:f>
+              <c:f>Sheet1!$B$16:$B$29</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2523,7 +2741,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$15:$F$28</c:f>
+              <c:f>Sheet1!$F$16:$F$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -2593,7 +2811,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$15:$B$28</c:f>
+              <c:f>Sheet1!$B$16:$B$29</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2604,7 +2822,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$15:$H$28</c:f>
+              <c:f>Sheet1!$H$16:$H$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -2671,7 +2889,7 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$J$15:$J$28</c:f>
+              <c:f>Sheet1!$J$16:$J$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -2952,279 +3170,8 @@
         <c:grouping val="standard"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="1"/>
+          <c:idx val="8"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$C$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>4 SE</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050">
-              <a:solidFill>
-                <a:schemeClr val="accent6"/>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Operational Runs</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$C$30:$C$43</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
-                <c:pt idx="9">
-                  <c:v>197</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>171</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>198</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>196</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>200</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-B1FF-4D4B-80A3-ACE12560F529}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$E$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>5 SE</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050">
-              <a:solidFill>
-                <a:schemeClr val="accent1">
-                  <a:lumMod val="60000"/>
-                  <a:lumOff val="40000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Operational Runs</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$E$30:$E$43</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
-                <c:pt idx="6">
-                  <c:v>72</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>71</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>62</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>72</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>77</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-B1FF-4D4B-80A3-ACE12560F529}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="4"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$G$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>6 SE</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050">
-              <a:solidFill>
-                <a:schemeClr val="accent4">
-                  <a:lumMod val="75000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Operational Runs</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$G$30:$G$43</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
-                <c:pt idx="5">
-                  <c:v>157</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>135</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>145</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>147</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>156</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000A-B1FF-4D4B-80A3-ACE12560F529}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="7"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Sheet1!$I$2</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>7 SE</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="19050">
-              <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:lumMod val="75000"/>
-                </a:schemeClr>
-              </a:solidFill>
-            </a:ln>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Operational Runs</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Sheet1!$I$30:$I$43</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="14"/>
-                <c:pt idx="6">
-                  <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>32</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>51</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>46</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000B-B1FF-4D4B-80A3-ACE12560F529}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="8"/>
-          <c:order val="4"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$D$2</c:f>
@@ -3250,7 +3197,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3261,7 +3208,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$30:$D$43</c:f>
+              <c:f>Sheet1!$D$31:$D$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -3292,7 +3239,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="9"/>
-          <c:order val="5"/>
+          <c:order val="1"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$F$2</c:f>
@@ -3320,7 +3267,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3331,7 +3278,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$30:$F$43</c:f>
+              <c:f>Sheet1!$F$31:$F$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -3362,7 +3309,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="10"/>
-          <c:order val="6"/>
+          <c:order val="2"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$H$2</c:f>
@@ -3386,7 +3333,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3397,7 +3344,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$30:$H$43</c:f>
+              <c:f>Sheet1!$H$31:$H$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -3428,7 +3375,7 @@
         </c:ser>
         <c:ser>
           <c:idx val="0"/>
-          <c:order val="7"/>
+          <c:order val="3"/>
           <c:tx>
             <c:strRef>
               <c:f>Sheet1!$J$2</c:f>
@@ -3452,7 +3399,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3463,7 +3410,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$J$30:$J$43</c:f>
+              <c:f>Sheet1!$J$31:$J$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -3489,6 +3436,332 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000007-B1FF-4D4B-80A3-ACE12560F529}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>4 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$31:$C$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="9">
+                  <c:v>197</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>171</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>198</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>196</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-B1FF-4D4B-80A3-ACE12560F529}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$E$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                  <a:lumOff val="40000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$E$31:$E$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="6">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>62</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>77</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000009-B1FF-4D4B-80A3-ACE12560F529}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$G$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$G$31:$G$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="5">
+                  <c:v>157</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>145</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>147</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>156</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000A-B1FF-4D4B-80A3-ACE12560F529}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="7"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$I$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$I$31:$I$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="6">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{0000000B-B1FF-4D4B-80A3-ACE12560F529}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="8"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$K$31:$K$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>48</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5436-4951-A04D-A204DB22F441}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3759,7 +4032,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3770,7 +4043,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$30:$C$43</c:f>
+              <c:f>Sheet1!$C$31:$C$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -3828,7 +4101,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3839,7 +4112,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$30:$E$43</c:f>
+              <c:f>Sheet1!$E$31:$E$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -3896,7 +4169,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3907,7 +4180,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$30:$G$43</c:f>
+              <c:f>Sheet1!$G$31:$G$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -3964,7 +4237,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3975,7 +4248,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$30:$I$43</c:f>
+              <c:f>Sheet1!$I$31:$I$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -4001,6 +4274,61 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000003-385B-4DAE-8633-EB08A908D7E0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$K$31:$K$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>48</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-CA77-442F-84A1-E7CE25432F06}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4274,7 +4602,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4285,7 +4613,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$30:$D$43</c:f>
+              <c:f>Sheet1!$D$31:$D$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -4344,7 +4672,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4355,7 +4683,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$30:$F$43</c:f>
+              <c:f>Sheet1!$F$31:$F$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -4410,7 +4738,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4421,7 +4749,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$30:$H$43</c:f>
+              <c:f>Sheet1!$H$31:$H$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -4476,7 +4804,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$B$29</c:f>
+              <c:f>Sheet1!$B$31</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4487,7 +4815,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$J$30:$J$43</c:f>
+              <c:f>Sheet1!$J$31:$J$44</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="14"/>
@@ -4585,6 +4913,640 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="300"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Distance</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> to wall (mm)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1430609439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst/>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="8"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$D$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>4 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$D$31:$D$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="8">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>97</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E24F-4D71-A167-9AB09D3CA728}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="9"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$F$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$F$31:$F$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="6">
+                  <c:v>193</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>257</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>183</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>180</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E24F-4D71-A167-9AB09D3CA728}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="10"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$H$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$H$31:$H$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="6">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>239</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>248</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>262</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-E24F-4D71-A167-9AB09D3CA728}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$J$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7 Freestyle</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:srgbClr val="994010"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$J$31:$J$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="5">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>184</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>176</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>179</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>185</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-E24F-4D71-A167-9AB09D3CA728}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="7"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$I$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>7 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$31</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Operational Runs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$I$31:$I$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="6">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-E24F-4D71-A167-9AB09D3CA728}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8 SE</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$K$31:$K$44</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="5">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>48</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-E24F-4D71-A167-9AB09D3CA728}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="1430609439"/>
+        <c:axId val="1430609919"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1430609439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1430609919"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:tickMarkSkip val="1"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1430609919"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -5828,7 +6790,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -5864,7 +6826,7 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -5873,7 +6835,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>29</xdr:row>
-      <xdr:rowOff>179293</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -5948,7 +6910,7 @@
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>29</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -5978,16 +6940,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>177390</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>3810</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6019,13 +6981,13 @@
       <xdr:col>18</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>175598</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>45</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>1792</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6057,13 +7019,13 @@
       <xdr:col>18</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>45</xdr:row>
-      <xdr:rowOff>175598</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>4649</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6085,6 +7047,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>6667</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Chart 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{811A54EE-129C-441A-917C-8A49D98F2579}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -6410,7 +7410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22FC483D-A2EB-4AB5-93A8-361DFBAB7337}">
-  <dimension ref="B2:K43"/>
+  <dimension ref="B2:L44"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.3984375" customWidth="1"/>
@@ -6419,12 +7419,12 @@
     <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="9.265625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="10" width="9.33203125" customWidth="1"/>
-    <col min="11" max="11" width="2.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="11" width="9.33203125" customWidth="1"/>
+    <col min="12" max="12" width="2.33203125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="2.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
@@ -6452,8 +7452,11 @@
       <c r="J2" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="K2" s="2" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
@@ -6481,9 +7484,12 @@
       <c r="J3" s="11">
         <v>46210</v>
       </c>
-      <c r="K3" s="10"/>
+      <c r="K3" s="11">
+        <v>46211</v>
+      </c>
+      <c r="L3" s="10"/>
     </row>
-    <row r="4" spans="2:11" s="15" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:12" s="15" customFormat="1" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
@@ -6509,9 +7515,12 @@
       <c r="J4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="14"/>
+      <c r="K4" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="L4" s="14"/>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
@@ -6539,9 +7548,12 @@
       <c r="J5" s="3">
         <v>4</v>
       </c>
-      <c r="K5" s="3"/>
+      <c r="K5" s="3">
+        <v>4</v>
+      </c>
+      <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B6" s="1" t="s">
         <v>25</v>
       </c>
@@ -6569,9 +7581,12 @@
       <c r="J6" s="3">
         <v>0</v>
       </c>
-      <c r="K6" s="3"/>
+      <c r="K6" s="3">
+        <v>1</v>
+      </c>
+      <c r="L6" s="3"/>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B7" s="1" t="s">
         <v>26</v>
       </c>
@@ -6599,9 +7614,12 @@
       <c r="J7" s="3">
         <v>1</v>
       </c>
-      <c r="K7" s="3"/>
+      <c r="K7" s="3">
+        <v>0</v>
+      </c>
+      <c r="L7" s="3"/>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B8" s="1" t="s">
         <v>1</v>
       </c>
@@ -6629,14 +7647,17 @@
       <c r="J8" s="3">
         <v>1</v>
       </c>
-      <c r="K8" s="3"/>
+      <c r="K8" s="3">
+        <v>1</v>
+      </c>
+      <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="7">
-        <f t="shared" ref="C9:J9" si="0">C8+C5</f>
+        <f t="shared" ref="C9:K9" si="0">C8+C5</f>
         <v>9</v>
       </c>
       <c r="D9" s="7">
@@ -6667,9 +7688,13 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="K9" s="3"/>
+      <c r="K9" s="7">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="L9" s="3"/>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B10" s="1" t="s">
         <v>2</v>
       </c>
@@ -6697,9 +7722,12 @@
       <c r="J10" s="4">
         <v>175.4</v>
       </c>
-      <c r="K10" s="4"/>
+      <c r="K10" s="4">
+        <v>43.4</v>
+      </c>
+      <c r="L10" s="4"/>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
@@ -6727,9 +7755,12 @@
       <c r="J11" s="5">
         <v>32</v>
       </c>
-      <c r="K11" s="5"/>
+      <c r="K11" s="5">
+        <v>19</v>
+      </c>
+      <c r="L11" s="5"/>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B12" s="1" t="s">
         <v>21</v>
       </c>
@@ -6757,9 +7788,12 @@
       <c r="J12" s="9">
         <v>13.049904214207857</v>
       </c>
-      <c r="K12" s="5"/>
+      <c r="K12" s="9">
+        <v>7.700649323271394</v>
+      </c>
+      <c r="L12" s="5"/>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B13" s="1" t="s">
         <v>10</v>
       </c>
@@ -6773,7 +7807,7 @@
         <v>78</v>
       </c>
       <c r="F13" s="5">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G13" s="5">
         <v>44</v>
@@ -6786,16 +7820,19 @@
         <v>55</v>
       </c>
       <c r="J13" s="5">
-        <v>42</v>
-      </c>
-      <c r="K13" s="5"/>
+        <v>45</v>
+      </c>
+      <c r="K13" s="5">
+        <v>45</v>
+      </c>
+      <c r="L13" s="5"/>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B14" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="9">
-        <f t="shared" ref="C14:J14" si="1">C10-C13</f>
+        <f t="shared" ref="C14:K14" si="1">C10-C13</f>
         <v>3.4000000000000057</v>
       </c>
       <c r="D14" s="9">
@@ -6808,7 +7845,7 @@
       </c>
       <c r="F14" s="9">
         <f t="shared" si="1"/>
-        <v>158.80000000000001</v>
+        <v>154.80000000000001</v>
       </c>
       <c r="G14" s="9">
         <f t="shared" si="1"/>
@@ -6824,542 +7861,627 @@
       </c>
       <c r="J14" s="9">
         <f t="shared" si="1"/>
-        <v>133.4</v>
-      </c>
-      <c r="K14" s="5"/>
+        <v>130.4</v>
+      </c>
+      <c r="K14" s="9">
+        <f t="shared" si="1"/>
+        <v>-1.6000000000000014</v>
+      </c>
+      <c r="L14" s="5"/>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B15" s="16" t="s">
+    <row r="15" spans="2:12" s="19" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="B15" s="17"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="18"/>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B16" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="3">
+      <c r="C16" s="3"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="3">
         <v>533</v>
       </c>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2">
+        <v>515</v>
+      </c>
+      <c r="L16" s="2"/>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B16" s="16"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2">
-        <v>442</v>
-      </c>
-      <c r="F16" s="2">
-        <v>228</v>
-      </c>
-      <c r="G16" s="3">
-        <v>498</v>
-      </c>
-      <c r="H16" s="3"/>
-      <c r="I16" s="2">
-        <v>196</v>
-      </c>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B17" s="16"/>
-      <c r="C17" s="3">
-        <v>314</v>
-      </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2">
-        <v>689</v>
+        <v>442</v>
       </c>
       <c r="F17" s="2">
-        <v>78</v>
+        <v>228</v>
       </c>
       <c r="G17" s="3">
-        <v>530</v>
-      </c>
-      <c r="H17" s="2">
-        <v>421</v>
-      </c>
+        <v>498</v>
+      </c>
+      <c r="H17" s="3"/>
       <c r="I17" s="2">
-        <v>113</v>
-      </c>
-      <c r="J17" s="2">
-        <v>345</v>
-      </c>
-      <c r="K17" s="2"/>
+        <v>196</v>
+      </c>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2">
+        <v>522</v>
+      </c>
+      <c r="L17" s="2"/>
     </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B18" s="16"/>
       <c r="C18" s="3">
-        <v>359</v>
+        <v>314</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2">
-        <v>479</v>
+        <v>689</v>
       </c>
       <c r="F18" s="2">
-        <v>191</v>
+        <v>78</v>
       </c>
       <c r="G18" s="3">
-        <v>138</v>
+        <v>530</v>
       </c>
       <c r="H18" s="2">
-        <v>224</v>
+        <v>421</v>
       </c>
       <c r="I18" s="2">
-        <v>138</v>
+        <v>113</v>
       </c>
       <c r="J18" s="2">
-        <v>338</v>
-      </c>
-      <c r="K18" s="2"/>
+        <v>345</v>
+      </c>
+      <c r="K18" s="2">
+        <v>513</v>
+      </c>
+      <c r="L18" s="2"/>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B19" s="16"/>
       <c r="C19" s="3">
-        <v>641</v>
+        <v>359</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2">
-        <v>264</v>
+        <v>479</v>
       </c>
       <c r="F19" s="2">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="G19" s="3">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="H19" s="2">
-        <v>809</v>
+        <v>224</v>
       </c>
       <c r="I19" s="2">
-        <v>28</v>
+        <v>138</v>
       </c>
       <c r="J19" s="2">
-        <v>212</v>
-      </c>
+        <v>338</v>
+      </c>
+      <c r="K19" s="2">
+        <v>542</v>
+      </c>
+      <c r="L19" s="2"/>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B20" s="16"/>
       <c r="C20" s="3">
-        <v>409</v>
-      </c>
-      <c r="D20" s="2">
-        <v>395</v>
-      </c>
+        <v>641</v>
+      </c>
+      <c r="D20" s="2"/>
       <c r="E20" s="2">
-        <v>74</v>
+        <v>264</v>
       </c>
       <c r="F20" s="2">
-        <v>201</v>
+        <v>178</v>
       </c>
       <c r="G20" s="3">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="H20" s="2">
-        <v>129</v>
+        <v>809</v>
       </c>
       <c r="I20" s="2">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="J20" s="2">
-        <v>153</v>
+        <v>212</v>
+      </c>
+      <c r="K20" s="2">
+        <v>33</v>
       </c>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B21" s="16"/>
       <c r="C21" s="3">
-        <v>366</v>
+        <v>409</v>
       </c>
       <c r="D21" s="2">
-        <v>33</v>
+        <v>395</v>
       </c>
       <c r="E21" s="2">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F21" s="2">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="G21" s="3">
-        <v>135</v>
+        <v>157</v>
       </c>
       <c r="H21" s="2">
-        <v>39</v>
+        <v>129</v>
       </c>
       <c r="I21" s="2">
         <v>46</v>
       </c>
       <c r="J21" s="2">
-        <v>184</v>
+        <v>153</v>
+      </c>
+      <c r="K21" s="2">
+        <v>31</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B22" s="16"/>
       <c r="C22" s="3">
-        <v>469</v>
+        <v>366</v>
       </c>
       <c r="D22" s="2">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="E22" s="2">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F22" s="2">
-        <v>257</v>
+        <v>193</v>
       </c>
       <c r="G22" s="3">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="H22" s="2">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="I22" s="2">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J22" s="2">
-        <v>176</v>
-      </c>
-      <c r="K22" s="2"/>
+        <v>184</v>
+      </c>
+      <c r="K22" s="2">
+        <v>47</v>
+      </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B23" s="16"/>
       <c r="C23" s="3">
-        <v>173</v>
+        <v>469</v>
       </c>
       <c r="D23" s="2">
-        <v>99</v>
+        <v>38</v>
       </c>
       <c r="E23" s="2">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="F23" s="2">
-        <v>183</v>
+        <v>257</v>
       </c>
       <c r="G23" s="3">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H23" s="2">
-        <v>239</v>
+        <v>49</v>
       </c>
       <c r="I23" s="2">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="J23" s="2">
-        <v>179</v>
-      </c>
-      <c r="K23" s="2"/>
+        <v>176</v>
+      </c>
+      <c r="K23" s="2">
+        <v>50</v>
+      </c>
+      <c r="L23" s="2"/>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B24" s="16"/>
       <c r="C24" s="3">
-        <v>197</v>
+        <v>173</v>
       </c>
       <c r="D24" s="2">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="E24" s="2">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="F24" s="2">
-        <v>256</v>
+        <v>183</v>
       </c>
       <c r="G24" s="3">
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="H24" s="2">
-        <v>248</v>
+        <v>239</v>
       </c>
       <c r="I24" s="2">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="J24" s="2">
-        <v>185</v>
-      </c>
-      <c r="K24" s="2"/>
+        <v>179</v>
+      </c>
+      <c r="K24" s="2">
+        <v>41</v>
+      </c>
+      <c r="L24" s="2"/>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B25" s="16"/>
       <c r="C25" s="3">
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D25" s="2">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E25" s="2">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F25" s="2">
-        <v>180</v>
-      </c>
-      <c r="G25" s="2"/>
+        <v>256</v>
+      </c>
+      <c r="G25" s="3">
+        <v>156</v>
+      </c>
       <c r="H25" s="2">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="I25" s="2">
-        <v>46</v>
-      </c>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
+        <v>51</v>
+      </c>
+      <c r="J25" s="2">
+        <v>185</v>
+      </c>
+      <c r="K25" s="2">
+        <v>48</v>
+      </c>
+      <c r="L25" s="2"/>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B26" s="16"/>
       <c r="C26" s="3">
-        <v>198</v>
+        <v>171</v>
       </c>
       <c r="D26" s="2">
-        <v>81</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="E26" s="2">
+        <v>77</v>
+      </c>
+      <c r="F26" s="2">
+        <v>180</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2">
+        <v>262</v>
+      </c>
+      <c r="I26" s="2">
+        <v>46</v>
+      </c>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
+      <c r="L26" s="2"/>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B27" s="16"/>
       <c r="C27" s="3">
+        <v>198</v>
+      </c>
+      <c r="D27" s="2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B28" s="16"/>
+      <c r="C28" s="3">
         <v>196</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D28" s="2">
         <v>97</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B28" s="16"/>
-      <c r="C28" s="7">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B29" s="16"/>
+      <c r="C29" s="7">
         <v>200</v>
       </c>
-      <c r="D28" s="6"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
     </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B29" s="16" t="s">
+    <row r="30" spans="2:12" s="19" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="B30" s="21"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="24"/>
+      <c r="I30" s="24"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="24"/>
+    </row>
+    <row r="31" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B31" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B30" s="16"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-    </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B31" s="16"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="5"/>
-    </row>
-    <row r="32" spans="2:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B32" s="16"/>
       <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="5"/>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B33" s="16"/>
       <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
     </row>
-    <row r="34" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B34" s="16"/>
       <c r="J34" s="2"/>
+      <c r="K34" s="2"/>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B35" s="16"/>
-      <c r="G35">
-        <f>G20</f>
-        <v>157</v>
-      </c>
-      <c r="J35" s="2">
-        <f>J20</f>
-        <v>153</v>
-      </c>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
     </row>
-    <row r="36" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B36" s="16"/>
-      <c r="E36">
-        <f t="shared" ref="E36:F40" si="2">E21</f>
-        <v>72</v>
-      </c>
-      <c r="F36">
-        <f t="shared" si="2"/>
-        <v>193</v>
-      </c>
       <c r="G36">
         <f>G21</f>
-        <v>135</v>
-      </c>
-      <c r="H36">
-        <f t="shared" ref="H36:I40" si="3">H21</f>
-        <v>39</v>
-      </c>
-      <c r="I36">
-        <f t="shared" si="3"/>
-        <v>46</v>
+        <v>157</v>
       </c>
       <c r="J36" s="2">
         <f>J21</f>
-        <v>184</v>
+        <v>153</v>
+      </c>
+      <c r="K36" s="2">
+        <f>K21</f>
+        <v>31</v>
       </c>
     </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B37" s="16"/>
       <c r="E37">
-        <f t="shared" si="2"/>
-        <v>71</v>
+        <f>E22</f>
+        <v>72</v>
       </c>
       <c r="F37">
-        <f t="shared" si="2"/>
-        <v>257</v>
+        <f>F22</f>
+        <v>193</v>
       </c>
       <c r="G37">
         <f>G22</f>
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="H37">
-        <f t="shared" si="3"/>
-        <v>49</v>
+        <f>H22</f>
+        <v>39</v>
       </c>
       <c r="I37">
-        <f t="shared" si="3"/>
-        <v>45</v>
+        <f>I22</f>
+        <v>46</v>
       </c>
       <c r="J37" s="2">
         <f>J22</f>
-        <v>176</v>
+        <v>184</v>
+      </c>
+      <c r="K37" s="2">
+        <f>K22</f>
+        <v>47</v>
       </c>
     </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B38" s="16"/>
-      <c r="D38">
-        <f>D23</f>
-        <v>99</v>
-      </c>
       <c r="E38">
-        <f t="shared" si="2"/>
-        <v>62</v>
+        <f>E23</f>
+        <v>71</v>
       </c>
       <c r="F38">
-        <f t="shared" si="2"/>
-        <v>183</v>
+        <f>F23</f>
+        <v>257</v>
       </c>
       <c r="G38">
         <f>G23</f>
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H38">
-        <f t="shared" si="3"/>
-        <v>239</v>
+        <f>H23</f>
+        <v>49</v>
       </c>
       <c r="I38">
-        <f t="shared" si="3"/>
-        <v>32</v>
+        <f>I23</f>
+        <v>45</v>
       </c>
       <c r="J38" s="2">
         <f>J23</f>
-        <v>179</v>
+        <v>176</v>
+      </c>
+      <c r="K38" s="2">
+        <f>K23</f>
+        <v>50</v>
       </c>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B39" s="16"/>
-      <c r="C39">
-        <f>C24</f>
-        <v>197</v>
-      </c>
       <c r="D39">
         <f>D24</f>
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="E39">
-        <f t="shared" si="2"/>
-        <v>72</v>
+        <f>E24</f>
+        <v>62</v>
       </c>
       <c r="F39">
-        <f t="shared" si="2"/>
-        <v>256</v>
+        <f>F24</f>
+        <v>183</v>
       </c>
       <c r="G39">
         <f>G24</f>
-        <v>156</v>
+        <v>147</v>
       </c>
       <c r="H39">
-        <f t="shared" si="3"/>
-        <v>248</v>
+        <f>H24</f>
+        <v>239</v>
       </c>
       <c r="I39">
-        <f t="shared" si="3"/>
-        <v>51</v>
+        <f>I24</f>
+        <v>32</v>
       </c>
       <c r="J39" s="2">
         <f>J24</f>
-        <v>185</v>
+        <v>179</v>
+      </c>
+      <c r="K39" s="2">
+        <f>K24</f>
+        <v>41</v>
       </c>
     </row>
-    <row r="40" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B40" s="16"/>
       <c r="C40">
         <f>C25</f>
-        <v>171</v>
+        <v>197</v>
       </c>
       <c r="D40">
         <f>D25</f>
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="E40">
-        <f t="shared" si="2"/>
-        <v>77</v>
+        <f>E25</f>
+        <v>72</v>
       </c>
       <c r="F40">
-        <f t="shared" si="2"/>
-        <v>180</v>
+        <f>F25</f>
+        <v>256</v>
+      </c>
+      <c r="G40">
+        <f>G25</f>
+        <v>156</v>
       </c>
       <c r="H40">
-        <f t="shared" si="3"/>
-        <v>262</v>
+        <f>H25</f>
+        <v>248</v>
       </c>
       <c r="I40">
-        <f t="shared" si="3"/>
-        <v>46</v>
+        <f>I25</f>
+        <v>51</v>
+      </c>
+      <c r="J40" s="2">
+        <f>J25</f>
+        <v>185</v>
+      </c>
+      <c r="K40" s="2">
+        <f>K25</f>
+        <v>48</v>
       </c>
     </row>
-    <row r="41" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B41" s="16"/>
       <c r="C41">
         <f>C26</f>
-        <v>198</v>
+        <v>171</v>
       </c>
       <c r="D41">
         <f>D26</f>
-        <v>81</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="E41">
+        <f>E26</f>
+        <v>77</v>
+      </c>
+      <c r="F41">
+        <f>F26</f>
+        <v>180</v>
+      </c>
+      <c r="H41">
+        <f>H26</f>
+        <v>262</v>
+      </c>
+      <c r="I41">
+        <f>I26</f>
+        <v>46</v>
+      </c>
+      <c r="K41" s="2"/>
     </row>
-    <row r="42" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.45">
       <c r="B42" s="16"/>
       <c r="C42">
         <f>C27</f>
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D42">
         <f>D27</f>
+        <v>81</v>
+      </c>
+      <c r="K42" s="2"/>
+    </row>
+    <row r="43" spans="2:11" x14ac:dyDescent="0.45">
+      <c r="B43" s="16"/>
+      <c r="C43">
+        <f>C28</f>
+        <v>196</v>
+      </c>
+      <c r="D43">
+        <f>D28</f>
         <v>97</v>
       </c>
+      <c r="K43" s="2"/>
     </row>
-    <row r="43" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B43" s="16"/>
-      <c r="C43" s="8">
-        <f>C28</f>
+    <row r="44" spans="2:11" x14ac:dyDescent="0.45">
+      <c r="B44" s="16"/>
+      <c r="C44" s="8">
+        <f>C29</f>
         <v>200</v>
       </c>
-      <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
-      <c r="J43" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8"/>
+      <c r="H44" s="8"/>
+      <c r="I44" s="8"/>
+      <c r="J44" s="8"/>
+      <c r="K44" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B15:B28"/>
-    <mergeCell ref="B29:B43"/>
+    <mergeCell ref="B16:B29"/>
+    <mergeCell ref="B31:B44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Updated readme captions, corrected typo in Summary, deprecated se_test_procedure.
</commit_message>
<xml_diff>
--- a/latest/Spike-SysML Summary.xlsx
+++ b/latest/Spike-SysML Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jarret\Documents\GitHub\Spike-SysML\development\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A5D7800-0F0D-456E-B955-C60D267966B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF6B3FB3-6662-4FF5-B3CF-63BB85D4B2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34452" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{67E81273-2DCB-4899-8B48-DD4215E033B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4067,7 +4067,7 @@
                   <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7399,7 +7399,7 @@
                   <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8080,7 +8080,7 @@
                   <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10101,7 +10101,7 @@
                   <c:v>36</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>36</c:v>
+                  <c:v>35</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -14867,6 +14867,7 @@
         <v>48</v>
       </c>
       <c r="L40" s="2">
+        <f>L25</f>
         <v>15</v>
       </c>
       <c r="M40" s="2">
@@ -14903,7 +14904,8 @@
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
       <c r="M41" s="2">
-        <v>36</v>
+        <f>M26</f>
+        <v>35</v>
       </c>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.45">

</xml_diff>